<commit_message>
new template instructions (Schedule Editor)
</commit_message>
<xml_diff>
--- a/template_instructions.xlsx
+++ b/template_instructions.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jenny\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jenny\Documents\Logikhaus - JN files\JN - PROJECTS\AI projects\PROJ Schedule Editor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30E92F07-4041-421F-9834-9A3DFBDFAB2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B929A87-06D1-4242-90F9-F2695A6643CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="146" xr2:uid="{B8682349-D862-4141-AD82-F124EA4F9224}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
     <t>Replace from this</t>
   </si>
@@ -64,10 +64,6 @@
 where the old text was</t>
   </si>
   <si>
-    <t>Fill in the yellow cells, wherever applicable.
-Words are case-sensitive</t>
-  </si>
-  <si>
     <t>Guide for users &gt;&gt;</t>
   </si>
   <si>
@@ -98,6 +94,28 @@
   </si>
   <si>
     <t>Dropdown list: 12.08 for main spec, 8.06 for extras</t>
+  </si>
+  <si>
+    <t>R01.2 Nickel silver</t>
+  </si>
+  <si>
+    <t>SS</t>
+  </si>
+  <si>
+    <t>R01.2 NOWY SREBRNY</t>
+  </si>
+  <si>
+    <t>BLOKADA TILTFIRST</t>
+  </si>
+  <si>
+    <t>TILT FIRST, TURN FUNCTION BLOCKED</t>
+  </si>
+  <si>
+    <t>Blokada rozwarcia do okuć TiltFirst</t>
+  </si>
+  <si>
+    <t>Fill in the yellow cells, wherever applicable. Delete any template examples if needed
+Words are case-sensitive</t>
   </si>
 </sst>
 </file>
@@ -147,15 +165,13 @@
       <family val="2"/>
     </font>
     <font>
-      <i/>
-      <sz val="10"/>
+      <sz val="8"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
-      <i/>
-      <sz val="8"/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -267,7 +283,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -315,25 +331,28 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -679,8 +698,8 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.28515625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="30" style="1" customWidth="1"/>
-    <col min="3" max="3" width="27" style="1" customWidth="1"/>
+    <col min="2" max="2" width="35.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" style="1" customWidth="1"/>
     <col min="4" max="4" width="21" style="1" customWidth="1"/>
     <col min="5" max="6" width="19.7109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="34.42578125" style="1" customWidth="1"/>
@@ -694,20 +713,20 @@
     </row>
     <row r="2" spans="1:7" s="3" customFormat="1" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" s="17" t="s">
+      <c r="B2" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="19"/>
+      <c r="D2" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="18"/>
-      <c r="G2" s="20" t="s">
+      <c r="E2" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="19"/>
+      <c r="G2" s="21" t="s">
         <v>6</v>
       </c>
     </row>
@@ -722,10 +741,10 @@
         <v>2</v>
       </c>
       <c r="E3" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="10" t="s">
         <v>10</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>11</v>
       </c>
       <c r="G3" s="12" t="s">
         <v>4</v>
@@ -733,10 +752,10 @@
     </row>
     <row r="4" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>13</v>
       </c>
       <c r="D4" s="5">
         <v>8.06</v>
@@ -746,8 +765,12 @@
       <c r="G4" s="5"/>
     </row>
     <row r="5" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
+      <c r="B5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>18</v>
+      </c>
       <c r="D5" s="5">
         <v>12.08</v>
       </c>
@@ -756,8 +779,12 @@
       <c r="G5" s="5"/>
     </row>
     <row r="6" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
+      <c r="B6" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>18</v>
+      </c>
       <c r="D6" s="5">
         <v>12.08</v>
       </c>
@@ -766,16 +793,22 @@
       <c r="G6" s="5"/>
     </row>
     <row r="7" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
+      <c r="B7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="5">
+        <v>8.06</v>
+      </c>
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
     </row>
     <row r="8" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
@@ -815,27 +848,29 @@
     </row>
     <row r="13" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="14" spans="1:7" s="2" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="D14" s="23"/>
+      <c r="D14" s="24"/>
     </row>
     <row r="15" spans="1:7" s="13" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="14" t="s">
         <v>3</v>
       </c>
       <c r="C15" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="D15" s="14" t="s">
-        <v>11</v>
-      </c>
     </row>
     <row r="16" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="5"/>
+      <c r="B16" s="17" t="s">
+        <v>22</v>
+      </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
     </row>
@@ -870,7 +905,7 @@
     </row>
     <row r="25" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="F25" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
@@ -889,11 +924,8 @@
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="C14:D14"/>
   </mergeCells>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4" xr:uid="{15EBA63B-AD4D-4BF7-B54A-88125FB0D7B0}">
-      <formula1>$F$29:$F$30</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F13 D5:D12" xr:uid="{8B9CD125-3FAF-4A4F-808E-99D045C7AE2F}">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F13 D4:D12" xr:uid="{8B9CD125-3FAF-4A4F-808E-99D045C7AE2F}">
       <formula1>$F$26:$F$27</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
last column deleted, also more rows added
</commit_message>
<xml_diff>
--- a/template_instructions.xlsx
+++ b/template_instructions.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jenny\Documents\Logikhaus - JN files\JN - PROJECTS\AI projects\PROJ Schedule Editor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jenny\Documents\Logikhaus - JN files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B929A87-06D1-4242-90F9-F2695A6643CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C4244CA-0179-41F3-99E0-44909ED72C05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="146" xr2:uid="{B8682349-D862-4141-AD82-F124EA4F9224}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
   <si>
     <t>Replace from this</t>
   </si>
@@ -53,15 +53,7 @@
     <t>Delete these words from PDF</t>
   </si>
   <si>
-    <t>Match new text to the font style (eg. Bold, italics) and align it with</t>
-  </si>
-  <si>
     <t>Replace words in Schedule PDF</t>
-  </si>
-  <si>
-    <t>eg. Alu-clad colour:
-Handle:
-where the old text was</t>
   </si>
   <si>
     <t>Guide for users &gt;&gt;</t>
@@ -114,7 +106,7 @@
     <t>Blokada rozwarcia do okuć TiltFirst</t>
   </si>
   <si>
-    <t>Fill in the yellow cells, wherever applicable. Delete any template examples if needed
+    <t>Fill in the yellow cells, wherever applicable. Delete any examples if needed
 Words are case-sensitive</t>
   </si>
 </sst>
@@ -165,13 +157,13 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="8"/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="9"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -197,7 +189,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -244,19 +236,6 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
       <right/>
       <top style="thin">
         <color indexed="64"/>
@@ -283,7 +262,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -316,44 +295,38 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -694,7 +667,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C80EEA1-27D5-449A-9629-F8CC5E12AA1F}">
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.28515625" style="1" customWidth="1"/>
@@ -702,35 +675,31 @@
     <col min="3" max="3" width="43.140625" style="1" customWidth="1"/>
     <col min="4" max="4" width="21" style="1" customWidth="1"/>
     <col min="5" max="6" width="19.7109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="34.42578125" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="1"/>
+    <col min="7" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B1" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="3" customFormat="1" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="15" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" s="3" customFormat="1" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="20" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" s="19"/>
-      <c r="G2" s="21" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" s="8" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="21"/>
+      <c r="D2" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="21"/>
+    </row>
+    <row r="3" spans="1:6" s="8" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="9" t="s">
         <v>0</v>
       </c>
@@ -741,180 +710,188 @@
         <v>2</v>
       </c>
       <c r="E3" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="C4" s="5" t="s">
         <v>10</v>
-      </c>
-      <c r="G3" s="12" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>12</v>
       </c>
       <c r="D4" s="5">
         <v>8.06</v>
       </c>
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-    </row>
-    <row r="5" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:6" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D5" s="5">
         <v>12.08</v>
       </c>
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-    </row>
-    <row r="6" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:6" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D6" s="5">
         <v>12.08</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-    </row>
-    <row r="7" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:6" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D7" s="5">
         <v>8.06</v>
       </c>
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-    </row>
-    <row r="8" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
+    </row>
+    <row r="8" spans="1:6" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-    </row>
-    <row r="9" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:6" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-    </row>
-    <row r="10" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:6" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-    </row>
-    <row r="11" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
+    </row>
+    <row r="11" spans="1:6" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-    </row>
-    <row r="12" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:6" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
       <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-    </row>
-    <row r="13" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:7" s="2" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="C14" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="D14" s="24"/>
-    </row>
-    <row r="15" spans="1:7" s="13" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="14" t="s">
+    </row>
+    <row r="13" spans="1:6" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+    </row>
+    <row r="14" spans="1:6" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+    </row>
+    <row r="15" spans="1:6" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+    </row>
+    <row r="16" spans="1:6" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="17" spans="1:6" s="2" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="19"/>
+    </row>
+    <row r="18" spans="1:6" s="12" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="C15" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="D15" s="14" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-    </row>
-    <row r="17" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-    </row>
-    <row r="18" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-    </row>
-    <row r="19" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="5"/>
+      <c r="C18" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="16" t="s">
+        <v>20</v>
+      </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
     </row>
-    <row r="20" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
       <c r="D20" s="5"/>
     </row>
-    <row r="21" spans="1:7" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A22"/>
-      <c r="B22"/>
-      <c r="C22"/>
-      <c r="D22"/>
-      <c r="E22"/>
-      <c r="G22"/>
-    </row>
-    <row r="25" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="F25" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="F26" s="1">
+    <row r="21" spans="1:6" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+    </row>
+    <row r="22" spans="1:6" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+    </row>
+    <row r="23" spans="1:6" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+    </row>
+    <row r="24" spans="1:6" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:6" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="A25"/>
+      <c r="B25"/>
+      <c r="C25"/>
+      <c r="D25"/>
+      <c r="E25"/>
+    </row>
+    <row r="28" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="F28" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F29" s="1">
         <v>12.08</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="F27" s="1">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F30" s="1">
         <v>8.06</v>
       </c>
     </row>
@@ -922,11 +899,11 @@
   <mergeCells count="3">
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
-    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C17:D17"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F13 D4:D12" xr:uid="{8B9CD125-3FAF-4A4F-808E-99D045C7AE2F}">
-      <formula1>$F$26:$F$27</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F16 D4:D15" xr:uid="{8B9CD125-3FAF-4A4F-808E-99D045C7AE2F}">
+      <formula1>$F$29:$F$30</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>